<commit_message>
add report date to sql tables and reset_data func
</commit_message>
<xml_diff>
--- a/balance_gen_add_data/input/dep_beh_models.xlsx
+++ b/balance_gen_add_data/input/dep_beh_models.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dzimi\Documents\data_engineering\data_projects\git_hub_projects\bank_project\balance_gen_add_data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ACD1AA8-399D-4A79-B363-B289B5CBDC33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BEE09C8-29E8-445C-9BE1-39BA8B454A29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="4395" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="203">
   <si>
     <t>tenor</t>
   </si>
@@ -642,6 +642,9 @@
   </si>
   <si>
     <t>200M</t>
+  </si>
+  <si>
+    <t>report_date</t>
   </si>
 </sst>
 </file>
@@ -686,9 +689,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -978,1568 +982,2173 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1">
+      <c r="C1" s="1">
         <v>6000</v>
       </c>
-      <c r="C1" s="1">
+      <c r="D1" s="1">
         <v>8000</v>
       </c>
-      <c r="D1" s="1">
+      <c r="E1" s="1">
         <v>7060</v>
       </c>
-      <c r="E1" s="1">
+      <c r="F1" s="1">
         <v>7030</v>
       </c>
-      <c r="F1" s="1">
+      <c r="G1" s="1">
         <v>7010</v>
       </c>
-      <c r="G1" s="1">
+      <c r="H1" s="1">
         <v>7120</v>
       </c>
-      <c r="H1" s="1"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B2" t="s">
         <v>1</v>
-      </c>
-      <c r="B2">
-        <v>0.8</v>
       </c>
       <c r="C2">
         <v>0.8</v>
       </c>
       <c r="D2">
-        <v>0.99</v>
+        <v>0.8</v>
       </c>
       <c r="E2">
         <v>0.99</v>
       </c>
       <c r="F2">
+        <v>0.99</v>
+      </c>
+      <c r="G2">
         <v>0.9</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>0.99</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="A3" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B3" t="s">
         <v>2</v>
-      </c>
-      <c r="B3">
-        <v>0.78</v>
       </c>
       <c r="C3">
         <v>0.78</v>
       </c>
       <c r="D3">
+        <v>0.78</v>
+      </c>
+      <c r="E3">
         <v>0.98</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>0.97</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>0.85</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>0.98</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="A4" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B4" t="s">
         <v>3</v>
-      </c>
-      <c r="B4">
-        <v>0.76</v>
       </c>
       <c r="C4">
         <v>0.76</v>
       </c>
       <c r="D4">
+        <v>0.76</v>
+      </c>
+      <c r="E4">
         <v>0.97</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <v>0.95</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>0.8</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>0.97</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="A5" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B5" t="s">
         <v>4</v>
-      </c>
-      <c r="B5">
-        <v>0.74</v>
       </c>
       <c r="C5">
         <v>0.74</v>
       </c>
       <c r="D5">
+        <v>0.74</v>
+      </c>
+      <c r="E5">
         <v>0.96</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>0.9</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>0.75</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>0.96</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="A6" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B6" t="s">
         <v>5</v>
-      </c>
-      <c r="B6">
-        <v>0.72</v>
       </c>
       <c r="C6">
         <v>0.72</v>
       </c>
       <c r="D6">
+        <v>0.72</v>
+      </c>
+      <c r="E6">
         <v>0.95</v>
       </c>
-      <c r="E6">
+      <c r="F6">
         <v>0.85</v>
       </c>
-      <c r="F6">
+      <c r="G6">
         <v>0.7</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>0.95</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+      <c r="A7" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B7" t="s">
         <v>6</v>
-      </c>
-      <c r="B7">
-        <v>0.7</v>
       </c>
       <c r="C7">
         <v>0.7</v>
       </c>
       <c r="D7">
+        <v>0.7</v>
+      </c>
+      <c r="E7">
         <v>0.94</v>
       </c>
-      <c r="E7">
+      <c r="F7">
         <v>0.8</v>
       </c>
-      <c r="F7">
+      <c r="G7">
         <v>0.65</v>
       </c>
-      <c r="G7">
+      <c r="H7">
         <v>0.94</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
+      <c r="A8" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B8" t="s">
         <v>7</v>
-      </c>
-      <c r="B8">
-        <v>0.68</v>
       </c>
       <c r="C8">
         <v>0.68</v>
       </c>
       <c r="D8">
+        <v>0.68</v>
+      </c>
+      <c r="E8">
         <v>0.93</v>
       </c>
-      <c r="E8">
+      <c r="F8">
         <v>0.75</v>
       </c>
-      <c r="F8">
+      <c r="G8">
         <v>0.6</v>
       </c>
-      <c r="G8">
+      <c r="H8">
         <v>0.93</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+      <c r="A9" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B9" t="s">
         <v>8</v>
-      </c>
-      <c r="B9">
-        <v>0.66</v>
       </c>
       <c r="C9">
         <v>0.66</v>
       </c>
       <c r="D9">
+        <v>0.66</v>
+      </c>
+      <c r="E9">
         <v>0.85</v>
       </c>
-      <c r="E9">
+      <c r="F9">
         <v>0.7</v>
       </c>
-      <c r="F9">
+      <c r="G9">
         <v>0.55000000000000004</v>
       </c>
-      <c r="G9">
+      <c r="H9">
         <v>0.92</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
+      <c r="A10" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B10" t="s">
         <v>9</v>
-      </c>
-      <c r="B10">
-        <v>0.64</v>
       </c>
       <c r="C10">
         <v>0.64</v>
       </c>
       <c r="D10">
+        <v>0.64</v>
+      </c>
+      <c r="E10">
         <v>0.8</v>
       </c>
-      <c r="E10">
+      <c r="F10">
         <v>0.65</v>
       </c>
-      <c r="F10">
+      <c r="G10">
         <v>0.5</v>
       </c>
-      <c r="G10">
+      <c r="H10">
         <v>0.91</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
+      <c r="A11" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B11" t="s">
         <v>10</v>
-      </c>
-      <c r="B11">
-        <v>0.62</v>
       </c>
       <c r="C11">
         <v>0.62</v>
       </c>
       <c r="D11">
+        <v>0.62</v>
+      </c>
+      <c r="E11">
         <v>0.75</v>
       </c>
-      <c r="E11">
+      <c r="F11">
         <v>0.6</v>
       </c>
-      <c r="F11">
+      <c r="G11">
         <v>0.45</v>
       </c>
-      <c r="G11">
+      <c r="H11">
         <v>0.9</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
+      <c r="A12" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B12" t="s">
         <v>11</v>
-      </c>
-      <c r="B12">
-        <v>0.6</v>
       </c>
       <c r="C12">
         <v>0.6</v>
       </c>
       <c r="D12">
+        <v>0.6</v>
+      </c>
+      <c r="E12">
         <v>0.7</v>
       </c>
-      <c r="E12">
+      <c r="F12">
         <v>0.55000000000000004</v>
       </c>
-      <c r="F12">
+      <c r="G12">
         <v>0.4</v>
       </c>
-      <c r="G12">
+      <c r="H12">
         <v>0.89</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
+      <c r="A13" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B13" t="s">
         <v>12</v>
-      </c>
-      <c r="B13">
-        <v>0.57999999999999996</v>
       </c>
       <c r="C13">
         <v>0.57999999999999996</v>
       </c>
       <c r="D13">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="E13">
         <v>0.65</v>
       </c>
-      <c r="E13">
+      <c r="F13">
         <v>0.5</v>
       </c>
-      <c r="F13">
+      <c r="G13">
         <v>0.35</v>
       </c>
-      <c r="G13">
+      <c r="H13">
         <v>0.88</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
+      <c r="A14" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B14" t="s">
         <v>13</v>
-      </c>
-      <c r="B14">
-        <v>0.56000000000000005</v>
       </c>
       <c r="C14">
         <v>0.56000000000000005</v>
       </c>
       <c r="D14">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="E14">
         <v>0.6</v>
       </c>
-      <c r="E14">
+      <c r="F14">
         <v>0.45</v>
       </c>
-      <c r="F14">
+      <c r="G14">
         <v>0.3</v>
       </c>
-      <c r="G14">
+      <c r="H14">
         <v>0.85</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
+      <c r="A15" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B15" t="s">
         <v>14</v>
-      </c>
-      <c r="B15">
-        <v>0.54</v>
       </c>
       <c r="C15">
         <v>0.54</v>
       </c>
       <c r="D15">
+        <v>0.54</v>
+      </c>
+      <c r="E15">
         <v>0.55000000000000004</v>
       </c>
-      <c r="E15">
+      <c r="F15">
         <v>0.4</v>
       </c>
-      <c r="F15">
+      <c r="G15">
         <v>0.25</v>
       </c>
-      <c r="G15">
+      <c r="H15">
         <v>0.8</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
+      <c r="A16" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B16" t="s">
         <v>15</v>
-      </c>
-      <c r="B16">
-        <v>0.52</v>
       </c>
       <c r="C16">
         <v>0.52</v>
       </c>
       <c r="D16">
+        <v>0.52</v>
+      </c>
+      <c r="E16">
         <v>0.5</v>
       </c>
-      <c r="E16">
+      <c r="F16">
         <v>0.35</v>
       </c>
-      <c r="F16">
+      <c r="G16">
         <v>0.2</v>
       </c>
-      <c r="G16">
+      <c r="H16">
         <v>0.75</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A17" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B17" t="s">
         <v>16</v>
-      </c>
-      <c r="B17">
-        <v>0.5</v>
       </c>
       <c r="C17">
         <v>0.5</v>
       </c>
       <c r="D17">
+        <v>0.5</v>
+      </c>
+      <c r="E17">
         <v>0.45</v>
       </c>
-      <c r="E17">
+      <c r="F17">
         <v>0.3</v>
       </c>
-      <c r="F17">
+      <c r="G17">
         <v>0.15</v>
       </c>
-      <c r="G17">
+      <c r="H17">
         <v>0.7</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A18" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B18" t="s">
         <v>17</v>
-      </c>
-      <c r="B18">
-        <v>0.48</v>
       </c>
       <c r="C18">
         <v>0.48</v>
       </c>
       <c r="D18">
+        <v>0.48</v>
+      </c>
+      <c r="E18">
         <v>0.4</v>
       </c>
-      <c r="E18">
+      <c r="F18">
         <v>0.25</v>
       </c>
-      <c r="F18">
+      <c r="G18">
         <v>0.1</v>
       </c>
-      <c r="G18">
+      <c r="H18">
         <v>0.65</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A19" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B19" t="s">
         <v>18</v>
-      </c>
-      <c r="B19">
-        <v>0.46</v>
       </c>
       <c r="C19">
         <v>0.46</v>
       </c>
       <c r="D19">
+        <v>0.46</v>
+      </c>
+      <c r="E19">
         <v>0.35</v>
       </c>
-      <c r="E19">
+      <c r="F19">
         <v>0.2</v>
       </c>
-      <c r="F19">
+      <c r="G19">
         <v>0.05</v>
       </c>
-      <c r="G19">
+      <c r="H19">
         <v>0.6</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A20" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B20" t="s">
         <v>19</v>
-      </c>
-      <c r="B20">
-        <v>0.44</v>
       </c>
       <c r="C20">
         <v>0.44</v>
       </c>
       <c r="D20">
+        <v>0.44</v>
+      </c>
+      <c r="E20">
         <v>0.3</v>
       </c>
-      <c r="E20">
+      <c r="F20">
         <v>0.15</v>
       </c>
-      <c r="F20">
+      <c r="G20">
         <v>0</v>
       </c>
-      <c r="G20">
+      <c r="H20">
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A21" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B21" t="s">
         <v>20</v>
-      </c>
-      <c r="B21">
-        <v>0.42</v>
       </c>
       <c r="C21">
         <v>0.42</v>
       </c>
       <c r="D21">
+        <v>0.42</v>
+      </c>
+      <c r="E21">
         <v>0.25</v>
       </c>
-      <c r="E21">
+      <c r="F21">
         <v>0.1</v>
       </c>
-      <c r="G21">
+      <c r="H21">
         <v>0.5</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A22" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B22" t="s">
         <v>21</v>
-      </c>
-      <c r="B22">
-        <v>0.4</v>
       </c>
       <c r="C22">
         <v>0.4</v>
       </c>
       <c r="D22">
+        <v>0.4</v>
+      </c>
+      <c r="E22">
         <v>0.2</v>
       </c>
-      <c r="E22">
+      <c r="F22">
         <v>0.05</v>
       </c>
-      <c r="G22">
+      <c r="H22">
         <v>0.45</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A23" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B23" t="s">
         <v>22</v>
-      </c>
-      <c r="B23">
-        <v>0.38</v>
       </c>
       <c r="C23">
         <v>0.38</v>
       </c>
       <c r="D23">
+        <v>0.38</v>
+      </c>
+      <c r="E23">
         <v>0.15</v>
       </c>
-      <c r="E23">
+      <c r="F23">
         <v>0</v>
       </c>
-      <c r="G23">
+      <c r="H23">
         <v>0.4</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A24" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B24" t="s">
         <v>23</v>
-      </c>
-      <c r="B24">
-        <v>0.36</v>
       </c>
       <c r="C24">
         <v>0.36</v>
       </c>
       <c r="D24">
+        <v>0.36</v>
+      </c>
+      <c r="E24">
         <v>0.1</v>
       </c>
-      <c r="G24">
+      <c r="H24">
         <v>0.35</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A25" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B25" t="s">
         <v>24</v>
-      </c>
-      <c r="B25">
-        <v>0.34</v>
       </c>
       <c r="C25">
         <v>0.34</v>
       </c>
       <c r="D25">
+        <v>0.34</v>
+      </c>
+      <c r="E25">
         <v>0.05</v>
       </c>
-      <c r="G25">
+      <c r="H25">
         <v>0.3</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A26" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B26" t="s">
         <v>25</v>
-      </c>
-      <c r="B26">
-        <v>0.32</v>
       </c>
       <c r="C26">
         <v>0.32</v>
       </c>
       <c r="D26">
+        <v>0.32</v>
+      </c>
+      <c r="E26">
         <v>0</v>
       </c>
-      <c r="G26">
+      <c r="H26">
         <v>0.25</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A27" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B27" t="s">
         <v>26</v>
-      </c>
-      <c r="B27">
-        <v>0.3</v>
       </c>
       <c r="C27">
         <v>0.3</v>
       </c>
-      <c r="G27">
+      <c r="D27">
+        <v>0.3</v>
+      </c>
+      <c r="H27">
         <v>0.2</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A28" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B28" t="s">
         <v>27</v>
-      </c>
-      <c r="B28">
-        <v>0.28000000000000003</v>
       </c>
       <c r="C28">
         <v>0.28000000000000003</v>
       </c>
-      <c r="G28">
+      <c r="D28">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="H28">
         <v>0.15</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A29" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B29" t="s">
         <v>28</v>
-      </c>
-      <c r="B29">
-        <v>0.26</v>
       </c>
       <c r="C29">
         <v>0.26</v>
       </c>
-      <c r="G29">
+      <c r="D29">
+        <v>0.26</v>
+      </c>
+      <c r="H29">
         <v>0.1</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A30" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B30" t="s">
         <v>29</v>
-      </c>
-      <c r="B30">
-        <v>0.24</v>
       </c>
       <c r="C30">
         <v>0.24</v>
       </c>
-      <c r="G30">
+      <c r="D30">
+        <v>0.24</v>
+      </c>
+      <c r="H30">
         <v>0.05</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A31" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B31" t="s">
         <v>30</v>
-      </c>
-      <c r="B31">
-        <v>0.22</v>
       </c>
       <c r="C31">
         <v>0.22</v>
       </c>
-      <c r="G31">
+      <c r="D31">
+        <v>0.22</v>
+      </c>
+      <c r="H31">
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A32" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B32" t="s">
         <v>31</v>
-      </c>
-      <c r="B32">
-        <v>0.2</v>
       </c>
       <c r="C32">
         <v>0.2</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
+      <c r="D32">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B33" t="s">
         <v>32</v>
-      </c>
-      <c r="B33">
-        <v>0.18</v>
       </c>
       <c r="C33">
         <v>0.18</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
+      <c r="D33">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A34" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B34" t="s">
         <v>33</v>
-      </c>
-      <c r="B34">
-        <v>0.16</v>
       </c>
       <c r="C34">
         <v>0.16</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
+      <c r="D34">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A35" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B35" t="s">
         <v>34</v>
-      </c>
-      <c r="B35">
-        <v>0.14000000000000001</v>
       </c>
       <c r="C35">
         <v>0.14000000000000001</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
+      <c r="D35">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A36" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B36" t="s">
         <v>35</v>
-      </c>
-      <c r="B36">
-        <v>0.12</v>
       </c>
       <c r="C36">
         <v>0.12</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
+      <c r="D36">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A37" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B37" t="s">
         <v>36</v>
-      </c>
-      <c r="B37">
-        <v>0.1</v>
       </c>
       <c r="C37">
         <v>0.1</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
+      <c r="D37">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A38" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B38" t="s">
         <v>37</v>
-      </c>
-      <c r="B38">
-        <v>0.08</v>
       </c>
       <c r="C38">
         <v>0.08</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
+      <c r="D38">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A39" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B39" t="s">
         <v>38</v>
-      </c>
-      <c r="B39">
-        <v>0.06</v>
       </c>
       <c r="C39">
         <v>0.06</v>
       </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
+      <c r="D39">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A40" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B40" t="s">
         <v>39</v>
-      </c>
-      <c r="B40">
-        <v>0.04</v>
       </c>
       <c r="C40">
         <v>0.04</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
+      <c r="D40">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A41" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B41" t="s">
         <v>40</v>
-      </c>
-      <c r="B41">
-        <v>0.02</v>
       </c>
       <c r="C41">
         <v>0.02</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
+      <c r="D41">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A42" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B42" t="s">
         <v>41</v>
-      </c>
-      <c r="B42">
-        <v>0</v>
       </c>
       <c r="C42">
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
+      <c r="D42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A43" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B43" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A44" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B44" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A45" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B45" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A46" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B46" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A47" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B47" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A48" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B48" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A49" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B49" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A50" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B50" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A51" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B51" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A52" t="s">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A52" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B52" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A53" t="s">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A53" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B53" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A54" t="s">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A54" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B54" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A55" t="s">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A55" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B55" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A56" t="s">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A56" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B56" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A57" t="s">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A57" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B57" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A58" t="s">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A58" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B58" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A59" t="s">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A59" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B59" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A60" t="s">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A60" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B60" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A61" t="s">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A61" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B61" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A62" t="s">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A62" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B62" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A63" t="s">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A63" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B63" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A64" t="s">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A64" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B64" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A65" t="s">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A65" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B65" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A66" t="s">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A66" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B66" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A67" t="s">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A67" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B67" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A68" t="s">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A68" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B68" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A69" t="s">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A69" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B69" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A70" t="s">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A70" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B70" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A71" t="s">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A71" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B71" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A72" t="s">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A72" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B72" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A73" t="s">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A73" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B73" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A74" t="s">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A74" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B74" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A75" t="s">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A75" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B75" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A76" t="s">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A76" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B76" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A77" t="s">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A77" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B77" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A78" t="s">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A78" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B78" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A79" t="s">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A79" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B79" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A80" t="s">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A80" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B80" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A81" t="s">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A81" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B81" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A82" t="s">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A82" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B82" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A83" t="s">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A83" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B83" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A84" t="s">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A84" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B84" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A85" t="s">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A85" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B85" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A86" t="s">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A86" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B86" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A87" t="s">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A87" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B87" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A88" t="s">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A88" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B88" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A89" t="s">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A89" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B89" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A90" t="s">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A90" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B90" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A91" t="s">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A91" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B91" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A92" t="s">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A92" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B92" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A93" t="s">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A93" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B93" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A94" t="s">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A94" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B94" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A95" t="s">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A95" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B95" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A96" t="s">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A96" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B96" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A97" t="s">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A97" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B97" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A98" t="s">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A98" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B98" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A99" t="s">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A99" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B99" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A100" t="s">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A100" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B100" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A101" t="s">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A101" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B101" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A102" t="s">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A102" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B102" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A103" t="s">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A103" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B103" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A104" t="s">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A104" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B104" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A105" t="s">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A105" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B105" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A106" t="s">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A106" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B106" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A107" t="s">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A107" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B107" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A108" t="s">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A108" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B108" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A109" t="s">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A109" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B109" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A110" t="s">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A110" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B110" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A111" t="s">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A111" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B111" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A112" t="s">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A112" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B112" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A113" t="s">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A113" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B113" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A114" t="s">
+    <row r="114" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A114" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B114" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A115" t="s">
+    <row r="115" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A115" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B115" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A116" t="s">
+    <row r="116" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A116" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B116" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A117" t="s">
+    <row r="117" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A117" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B117" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A118" t="s">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A118" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B118" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A119" t="s">
+    <row r="119" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A119" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B119" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A120" t="s">
+    <row r="120" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A120" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B120" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A121" t="s">
+    <row r="121" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A121" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B121" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A122" t="s">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A122" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B122" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A123" t="s">
+    <row r="123" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A123" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B123" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A124" t="s">
+    <row r="124" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A124" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B124" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A125" t="s">
+    <row r="125" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A125" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B125" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A126" t="s">
+    <row r="126" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A126" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B126" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A127" t="s">
+    <row r="127" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A127" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B127" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A128" t="s">
+    <row r="128" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A128" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B128" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A129" t="s">
+    <row r="129" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A129" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B129" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="130" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A130" t="s">
+    <row r="130" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A130" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B130" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="131" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A131" t="s">
+    <row r="131" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A131" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B131" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="132" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A132" t="s">
+    <row r="132" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A132" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B132" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="133" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A133" t="s">
+    <row r="133" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A133" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B133" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="134" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A134" t="s">
+    <row r="134" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A134" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B134" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="135" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A135" t="s">
+    <row r="135" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A135" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B135" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="136" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A136" t="s">
+    <row r="136" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A136" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B136" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="137" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A137" t="s">
+    <row r="137" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A137" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B137" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="138" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A138" t="s">
+    <row r="138" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A138" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B138" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="139" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A139" t="s">
+    <row r="139" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A139" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B139" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="140" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A140" t="s">
+    <row r="140" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A140" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B140" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="141" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A141" t="s">
+    <row r="141" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A141" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B141" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="142" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A142" t="s">
+    <row r="142" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A142" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B142" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="143" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A143" t="s">
+    <row r="143" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A143" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B143" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="144" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A144" t="s">
+    <row r="144" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A144" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B144" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="145" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A145" t="s">
+    <row r="145" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A145" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B145" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="146" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A146" t="s">
+    <row r="146" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A146" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B146" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="147" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A147" t="s">
+    <row r="147" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A147" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B147" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="148" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A148" t="s">
+    <row r="148" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A148" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B148" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="149" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A149" t="s">
+    <row r="149" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A149" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B149" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="150" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A150" t="s">
+    <row r="150" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A150" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B150" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="151" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A151" t="s">
+    <row r="151" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A151" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B151" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="152" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A152" t="s">
+    <row r="152" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A152" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B152" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="153" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A153" t="s">
+    <row r="153" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A153" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B153" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="154" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A154" t="s">
+    <row r="154" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A154" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B154" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="155" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A155" t="s">
+    <row r="155" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A155" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B155" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="156" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A156" t="s">
+    <row r="156" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A156" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B156" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="157" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A157" t="s">
+    <row r="157" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A157" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B157" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="158" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A158" t="s">
+    <row r="158" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A158" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B158" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="159" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A159" t="s">
+    <row r="159" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A159" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B159" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="160" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A160" t="s">
+    <row r="160" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A160" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B160" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="161" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A161" t="s">
+    <row r="161" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A161" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B161" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="162" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A162" t="s">
+    <row r="162" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A162" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B162" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="163" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A163" t="s">
+    <row r="163" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A163" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B163" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="164" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A164" t="s">
+    <row r="164" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A164" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B164" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="165" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A165" t="s">
+    <row r="165" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A165" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B165" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="166" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A166" t="s">
+    <row r="166" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A166" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B166" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="167" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A167" t="s">
+    <row r="167" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A167" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B167" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="168" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A168" t="s">
+    <row r="168" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A168" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B168" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="169" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A169" t="s">
+    <row r="169" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A169" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B169" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="170" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A170" t="s">
+    <row r="170" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A170" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B170" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="171" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A171" t="s">
+    <row r="171" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A171" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B171" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="172" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A172" t="s">
+    <row r="172" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A172" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B172" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="173" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A173" t="s">
+    <row r="173" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A173" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B173" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="174" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A174" t="s">
+    <row r="174" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A174" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B174" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="175" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A175" t="s">
+    <row r="175" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A175" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B175" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="176" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A176" t="s">
+    <row r="176" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A176" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B176" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="177" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A177" t="s">
+    <row r="177" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A177" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B177" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="178" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A178" t="s">
+    <row r="178" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A178" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B178" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="179" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A179" t="s">
+    <row r="179" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A179" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B179" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="180" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A180" t="s">
+    <row r="180" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A180" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B180" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="181" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A181" t="s">
+    <row r="181" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A181" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B181" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="182" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A182" t="s">
+    <row r="182" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A182" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B182" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="183" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A183" t="s">
+    <row r="183" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A183" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B183" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="184" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A184" t="s">
+    <row r="184" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A184" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B184" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="185" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A185" t="s">
+    <row r="185" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A185" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B185" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="186" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A186" t="s">
+    <row r="186" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A186" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B186" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="187" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A187" t="s">
+    <row r="187" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A187" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B187" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="188" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A188" t="s">
+    <row r="188" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A188" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B188" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="189" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A189" t="s">
+    <row r="189" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A189" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B189" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="190" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A190" t="s">
+    <row r="190" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A190" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B190" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="191" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A191" t="s">
+    <row r="191" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A191" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B191" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="192" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A192" t="s">
+    <row r="192" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A192" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B192" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="193" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A193" t="s">
+    <row r="193" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A193" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B193" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="194" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A194" t="s">
+    <row r="194" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A194" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B194" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="195" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A195" t="s">
+    <row r="195" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A195" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B195" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="196" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A196" t="s">
+    <row r="196" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A196" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B196" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="197" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A197" t="s">
+    <row r="197" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A197" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B197" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="198" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A198" t="s">
+    <row r="198" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A198" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B198" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="199" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A199" t="s">
+    <row r="199" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A199" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B199" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="200" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A200" t="s">
+    <row r="200" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A200" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B200" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="201" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A201" t="s">
+    <row r="201" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A201" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B201" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="202" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A202" t="s">
+    <row r="202" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A202" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B202" t="s">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add lcr and nsfr calculation, also all irrbb shocks
</commit_message>
<xml_diff>
--- a/balance_gen_add_data/input/dep_beh_models.xlsx
+++ b/balance_gen_add_data/input/dep_beh_models.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dzimi\Documents\data_engineering\data_projects\git_hub_projects\bank_project\balance_gen_add_data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BEE09C8-29E8-445C-9BE1-39BA8B454A29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC2B8D63-4883-4F9C-AD28-AB53415DAC90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1174,7 +1174,7 @@
         <v>7</v>
       </c>
       <c r="C8">
-        <v>0.68</v>
+        <v>0.69</v>
       </c>
       <c r="D8">
         <v>0.68</v>
@@ -1200,7 +1200,7 @@
         <v>8</v>
       </c>
       <c r="C9">
-        <v>0.66</v>
+        <v>0.68</v>
       </c>
       <c r="D9">
         <v>0.66</v>
@@ -1226,7 +1226,7 @@
         <v>9</v>
       </c>
       <c r="C10">
-        <v>0.64</v>
+        <v>0.67</v>
       </c>
       <c r="D10">
         <v>0.64</v>
@@ -1252,7 +1252,7 @@
         <v>10</v>
       </c>
       <c r="C11">
-        <v>0.62</v>
+        <v>0.66</v>
       </c>
       <c r="D11">
         <v>0.62</v>
@@ -1278,7 +1278,7 @@
         <v>11</v>
       </c>
       <c r="C12">
-        <v>0.6</v>
+        <v>0.65</v>
       </c>
       <c r="D12">
         <v>0.6</v>
@@ -1304,7 +1304,7 @@
         <v>12</v>
       </c>
       <c r="C13">
-        <v>0.57999999999999996</v>
+        <v>0.64</v>
       </c>
       <c r="D13">
         <v>0.57999999999999996</v>
@@ -1330,7 +1330,7 @@
         <v>13</v>
       </c>
       <c r="C14">
-        <v>0.56000000000000005</v>
+        <v>0.63</v>
       </c>
       <c r="D14">
         <v>0.56000000000000005</v>
@@ -1356,7 +1356,7 @@
         <v>14</v>
       </c>
       <c r="C15">
-        <v>0.54</v>
+        <v>0.62</v>
       </c>
       <c r="D15">
         <v>0.54</v>
@@ -1382,7 +1382,7 @@
         <v>15</v>
       </c>
       <c r="C16">
-        <v>0.52</v>
+        <v>0.61</v>
       </c>
       <c r="D16">
         <v>0.52</v>
@@ -1408,7 +1408,7 @@
         <v>16</v>
       </c>
       <c r="C17">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="D17">
         <v>0.5</v>
@@ -1434,7 +1434,7 @@
         <v>17</v>
       </c>
       <c r="C18">
-        <v>0.48</v>
+        <v>0.59</v>
       </c>
       <c r="D18">
         <v>0.48</v>
@@ -1460,7 +1460,7 @@
         <v>18</v>
       </c>
       <c r="C19">
-        <v>0.46</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="D19">
         <v>0.46</v>
@@ -1486,7 +1486,7 @@
         <v>19</v>
       </c>
       <c r="C20">
-        <v>0.44</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="D20">
         <v>0.44</v>
@@ -1512,7 +1512,7 @@
         <v>20</v>
       </c>
       <c r="C21">
-        <v>0.42</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="D21">
         <v>0.42</v>
@@ -1535,7 +1535,7 @@
         <v>21</v>
       </c>
       <c r="C22">
-        <v>0.4</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="D22">
         <v>0.4</v>
@@ -1558,7 +1558,7 @@
         <v>22</v>
       </c>
       <c r="C23">
-        <v>0.38</v>
+        <v>0.54</v>
       </c>
       <c r="D23">
         <v>0.38</v>
@@ -1581,7 +1581,7 @@
         <v>23</v>
       </c>
       <c r="C24">
-        <v>0.36</v>
+        <v>0.53</v>
       </c>
       <c r="D24">
         <v>0.36</v>
@@ -1601,7 +1601,7 @@
         <v>24</v>
       </c>
       <c r="C25">
-        <v>0.34</v>
+        <v>0.52</v>
       </c>
       <c r="D25">
         <v>0.34</v>
@@ -1621,7 +1621,7 @@
         <v>25</v>
       </c>
       <c r="C26">
-        <v>0.32</v>
+        <v>0.51</v>
       </c>
       <c r="D26">
         <v>0.32</v>
@@ -1641,7 +1641,7 @@
         <v>26</v>
       </c>
       <c r="C27">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="D27">
         <v>0.3</v>
@@ -1658,7 +1658,7 @@
         <v>27</v>
       </c>
       <c r="C28">
-        <v>0.28000000000000003</v>
+        <v>0.49</v>
       </c>
       <c r="D28">
         <v>0.28000000000000003</v>
@@ -1675,7 +1675,7 @@
         <v>28</v>
       </c>
       <c r="C29">
-        <v>0.26</v>
+        <v>0.48</v>
       </c>
       <c r="D29">
         <v>0.26</v>
@@ -1692,7 +1692,7 @@
         <v>29</v>
       </c>
       <c r="C30">
-        <v>0.24</v>
+        <v>0.47</v>
       </c>
       <c r="D30">
         <v>0.24</v>
@@ -1709,7 +1709,7 @@
         <v>30</v>
       </c>
       <c r="C31">
-        <v>0.22</v>
+        <v>0.46</v>
       </c>
       <c r="D31">
         <v>0.22</v>
@@ -1726,7 +1726,7 @@
         <v>31</v>
       </c>
       <c r="C32">
-        <v>0.2</v>
+        <v>0.45</v>
       </c>
       <c r="D32">
         <v>0.2</v>
@@ -1740,7 +1740,7 @@
         <v>32</v>
       </c>
       <c r="C33">
-        <v>0.18</v>
+        <v>0.44</v>
       </c>
       <c r="D33">
         <v>0.18</v>
@@ -1754,7 +1754,7 @@
         <v>33</v>
       </c>
       <c r="C34">
-        <v>0.16</v>
+        <v>0.43</v>
       </c>
       <c r="D34">
         <v>0.16</v>
@@ -1768,7 +1768,7 @@
         <v>34</v>
       </c>
       <c r="C35">
-        <v>0.14000000000000001</v>
+        <v>0.42</v>
       </c>
       <c r="D35">
         <v>0.14000000000000001</v>
@@ -1782,7 +1782,7 @@
         <v>35</v>
       </c>
       <c r="C36">
-        <v>0.12</v>
+        <v>0.41</v>
       </c>
       <c r="D36">
         <v>0.12</v>
@@ -1796,7 +1796,7 @@
         <v>36</v>
       </c>
       <c r="C37">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="D37">
         <v>0.1</v>
@@ -1810,7 +1810,7 @@
         <v>37</v>
       </c>
       <c r="C38">
-        <v>0.08</v>
+        <v>0.39</v>
       </c>
       <c r="D38">
         <v>0.08</v>
@@ -1824,7 +1824,7 @@
         <v>38</v>
       </c>
       <c r="C39">
-        <v>0.06</v>
+        <v>0.38</v>
       </c>
       <c r="D39">
         <v>0.06</v>
@@ -1838,7 +1838,7 @@
         <v>39</v>
       </c>
       <c r="C40">
-        <v>0.04</v>
+        <v>0.37</v>
       </c>
       <c r="D40">
         <v>0.04</v>
@@ -1852,7 +1852,7 @@
         <v>40</v>
       </c>
       <c r="C41">
-        <v>0.02</v>
+        <v>0.36</v>
       </c>
       <c r="D41">
         <v>0.02</v>
@@ -1866,7 +1866,7 @@
         <v>41</v>
       </c>
       <c r="C42">
-        <v>0</v>
+        <v>0.35</v>
       </c>
       <c r="D42">
         <v>0</v>
@@ -1879,6 +1879,9 @@
       <c r="B43" t="s">
         <v>42</v>
       </c>
+      <c r="C43">
+        <v>0.34</v>
+      </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" s="2">
@@ -1887,6 +1890,9 @@
       <c r="B44" t="s">
         <v>43</v>
       </c>
+      <c r="C44">
+        <v>0.33</v>
+      </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" s="2">
@@ -1895,6 +1901,9 @@
       <c r="B45" t="s">
         <v>44</v>
       </c>
+      <c r="C45">
+        <v>0.32</v>
+      </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" s="2">
@@ -1903,6 +1912,9 @@
       <c r="B46" t="s">
         <v>45</v>
       </c>
+      <c r="C46">
+        <v>0.31</v>
+      </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" s="2">
@@ -1911,6 +1923,9 @@
       <c r="B47" t="s">
         <v>46</v>
       </c>
+      <c r="C47">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" s="2">
@@ -1919,240 +1934,330 @@
       <c r="B48" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C48">
+        <v>0.28999999999999998</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" s="2">
         <v>45657</v>
       </c>
       <c r="B49" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C49">
+        <v>0.28000000000000003</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" s="2">
         <v>45657</v>
       </c>
       <c r="B50" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C50">
+        <v>0.27</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" s="2">
         <v>45657</v>
       </c>
       <c r="B51" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C51">
+        <v>0.26</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" s="2">
         <v>45657</v>
       </c>
       <c r="B52" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C52">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" s="2">
         <v>45657</v>
       </c>
       <c r="B53" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C53">
+        <v>0.24</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A54" s="2">
         <v>45657</v>
       </c>
       <c r="B54" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C54">
+        <v>0.23</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A55" s="2">
         <v>45657</v>
       </c>
       <c r="B55" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C55">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A56" s="2">
         <v>45657</v>
       </c>
       <c r="B56" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C56">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A57" s="2">
         <v>45657</v>
       </c>
       <c r="B57" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C57">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A58" s="2">
         <v>45657</v>
       </c>
       <c r="B58" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C58">
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A59" s="2">
         <v>45657</v>
       </c>
       <c r="B59" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C59">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A60" s="2">
         <v>45657</v>
       </c>
       <c r="B60" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C60">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A61" s="2">
         <v>45657</v>
       </c>
       <c r="B61" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C61">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A62" s="2">
         <v>45657</v>
       </c>
       <c r="B62" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C62">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A63" s="2">
         <v>45657</v>
       </c>
       <c r="B63" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C63">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A64" s="2">
         <v>45657</v>
       </c>
       <c r="B64" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C64">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A65" s="2">
         <v>45657</v>
       </c>
       <c r="B65" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C65">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A66" s="2">
         <v>45657</v>
       </c>
       <c r="B66" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C66">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A67" s="2">
         <v>45657</v>
       </c>
       <c r="B67" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C67">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A68" s="2">
         <v>45657</v>
       </c>
       <c r="B68" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C68">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A69" s="2">
         <v>45657</v>
       </c>
       <c r="B69" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C69">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A70" s="2">
         <v>45657</v>
       </c>
       <c r="B70" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C70">
+        <v>7.0000000000000007E-2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A71" s="2">
         <v>45657</v>
       </c>
       <c r="B71" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C71">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A72" s="2">
         <v>45657</v>
       </c>
       <c r="B72" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C72">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A73" s="2">
         <v>45657</v>
       </c>
       <c r="B73" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C73">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A74" s="2">
         <v>45657</v>
       </c>
       <c r="B74" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C74">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A75" s="2">
         <v>45657</v>
       </c>
       <c r="B75" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C75">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A76" s="2">
         <v>45657</v>
       </c>
       <c r="B76" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C76">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A77" s="2">
         <v>45657</v>
       </c>
       <c r="B77" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C77">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A78" s="2">
         <v>45657</v>
       </c>
@@ -2160,7 +2265,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A79" s="2">
         <v>45657</v>
       </c>
@@ -2168,7 +2273,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A80" s="2">
         <v>45657</v>
       </c>

</xml_diff>